<commit_message>
Flujo completo de complementos de pago
</commit_message>
<xml_diff>
--- a/data/conceptos-escenario-ppd-1.xlsx
+++ b/data/conceptos-escenario-ppd-1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ErickAlejandroRodríg\Desktop\Entorno\FACTO\cfdi-automation\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF79EAE3-D305-404B-8650-47EACF4CDA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E6E87E3-2747-4303-82F8-582DF391BEA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-1515" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="escenarios" sheetId="1" r:id="rId1"/>
@@ -477,7 +477,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -602,8 +602,7 @@
     <xf numFmtId="0" fontId="0" fillId="20" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4304,7 +4303,6 @@
       <c r="H17" s="17">
         <v>220.17500000000001</v>
       </c>
-      <c r="J17" s="42"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="18">
@@ -4331,7 +4329,7 @@
       <c r="H18" s="18">
         <v>100</v>
       </c>
-      <c r="J18" s="43"/>
+      <c r="J18" s="42"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="19">
@@ -4358,7 +4356,6 @@
       <c r="H19" s="19">
         <v>98.92</v>
       </c>
-      <c r="J19" s="42"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="20">
@@ -4432,10 +4429,10 @@
         <v>5.7142999999999999E-2</v>
       </c>
       <c r="G22" s="22">
-        <v>1750</v>
+        <v>875</v>
       </c>
       <c r="H22" s="22">
-        <v>263</v>
+        <v>875</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
@@ -4458,10 +4455,10 @@
         <v>5.7142999999999999E-2</v>
       </c>
       <c r="G23" s="23">
-        <v>1750</v>
+        <v>875</v>
       </c>
       <c r="H23" s="23">
-        <v>110</v>
+        <v>875</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
estabilidad y correccion de matriz
</commit_message>
<xml_diff>
--- a/data/conceptos-escenario-ppd-1.xlsx
+++ b/data/conceptos-escenario-ppd-1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ErickAlejandroRodríg\Desktop\Entorno\FACTO\cfdi-automation\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E6E87E3-2747-4303-82F8-582DF391BEA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD7605D3-243F-46D4-9885-656DA0FAA15F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="escenarios" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="98">
   <si>
     <t>Id Escenario</t>
   </si>
@@ -149,9 +149,6 @@
     <t>Valor Unitario</t>
   </si>
   <si>
-    <t>Objeto Impuesto</t>
-  </si>
-  <si>
     <t>Servicio de prueba</t>
   </si>
   <si>
@@ -306,13 +303,40 @@
   </si>
   <si>
     <t>IVA 16 IVA 8 IVA 0 IEPS 0.53 IEPS 0.265 Ret IEPS 0.53 Ret ISR 0.15 Ret ISH 0.08</t>
+  </si>
+  <si>
+    <t>CP3</t>
+  </si>
+  <si>
+    <t>CP4</t>
+  </si>
+  <si>
+    <t>CP5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IVA 16 USD </t>
+  </si>
+  <si>
+    <t>IVA 16 USD</t>
+  </si>
+  <si>
+    <t>04</t>
+  </si>
+  <si>
+    <t>20/03/2027</t>
+  </si>
+  <si>
+    <t>20/03/2028</t>
+  </si>
+  <si>
+    <t>20/03/2029</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -325,6 +349,12 @@
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="25">
@@ -477,7 +507,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -602,7 +632,10 @@
     <xf numFmtId="0" fontId="0" fillId="20" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -907,7 +940,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1189,7 +1222,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C19" s="19" t="s">
         <v>17</v>
@@ -1254,14 +1287,63 @@
         <v>29</v>
       </c>
     </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A25" s="3">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A26" s="4">
+        <v>25</v>
+      </c>
+      <c r="B26" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A27" s="5">
+        <v>26</v>
+      </c>
+      <c r="B27" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1296,9 +1378,7 @@
       <c r="G1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>37</v>
-      </c>
+      <c r="H1" s="1"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
@@ -1311,19 +1391,19 @@
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="24" t="s">
         <v>87</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F2" s="24" t="s">
-        <v>88</v>
       </c>
       <c r="G2" s="2">
         <v>100</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
@@ -1337,19 +1417,19 @@
         <v>1</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" s="25" t="s">
         <v>87</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F3" s="25" t="s">
-        <v>88</v>
       </c>
       <c r="G3" s="3">
         <v>100</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -1363,19 +1443,19 @@
         <v>1</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" s="26" t="s">
         <v>87</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F4" s="26" t="s">
-        <v>88</v>
       </c>
       <c r="G4" s="4">
         <v>100</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -1389,19 +1469,19 @@
         <v>1</v>
       </c>
       <c r="D5" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" s="27" t="s">
         <v>87</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="F5" s="27" t="s">
-        <v>88</v>
       </c>
       <c r="G5" s="5">
         <v>100</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -1415,19 +1495,19 @@
         <v>1</v>
       </c>
       <c r="D6" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6" s="28" t="s">
         <v>87</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="F6" s="28" t="s">
-        <v>88</v>
       </c>
       <c r="G6" s="6">
         <v>100</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -1441,19 +1521,19 @@
         <v>1</v>
       </c>
       <c r="D7" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" s="29" t="s">
         <v>87</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="F7" s="29" t="s">
-        <v>88</v>
       </c>
       <c r="G7" s="7">
         <v>100</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
@@ -1467,19 +1547,19 @@
         <v>1</v>
       </c>
       <c r="D8" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="30" t="s">
         <v>87</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="F8" s="30" t="s">
-        <v>88</v>
       </c>
       <c r="G8" s="8">
         <v>100</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
@@ -1493,19 +1573,19 @@
         <v>1</v>
       </c>
       <c r="D9" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" s="31" t="s">
         <v>87</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="F9" s="31" t="s">
-        <v>88</v>
       </c>
       <c r="G9" s="9">
         <v>100</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
@@ -1519,19 +1599,19 @@
         <v>1</v>
       </c>
       <c r="D10" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="F10" s="32" t="s">
         <v>87</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="F10" s="32" t="s">
-        <v>88</v>
       </c>
       <c r="G10" s="10">
         <v>350</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
@@ -1545,19 +1625,19 @@
         <v>1</v>
       </c>
       <c r="D11" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="F11" s="33" t="s">
         <v>87</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="F11" s="33" t="s">
-        <v>88</v>
       </c>
       <c r="G11" s="11">
         <v>100</v>
       </c>
       <c r="H11" s="11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -1571,19 +1651,19 @@
         <v>1</v>
       </c>
       <c r="D12" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="F12" s="34" t="s">
         <v>87</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="F12" s="34" t="s">
-        <v>88</v>
       </c>
       <c r="G12" s="12">
         <v>100</v>
       </c>
       <c r="H12" s="12" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
@@ -1597,19 +1677,19 @@
         <v>1</v>
       </c>
       <c r="D13" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" s="35" t="s">
         <v>87</v>
-      </c>
-      <c r="E13" s="13" t="s">
-        <v>38</v>
-      </c>
-      <c r="F13" s="35" t="s">
-        <v>88</v>
       </c>
       <c r="G13" s="13">
         <v>100</v>
       </c>
       <c r="H13" s="13" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
@@ -1623,19 +1703,19 @@
         <v>1</v>
       </c>
       <c r="D14" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="F14" s="36" t="s">
         <v>87</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="F14" s="36" t="s">
-        <v>88</v>
       </c>
       <c r="G14" s="14">
         <v>117.43</v>
       </c>
       <c r="H14" s="14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
@@ -1649,19 +1729,19 @@
         <v>1</v>
       </c>
       <c r="D15" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="F15" s="37" t="s">
         <v>87</v>
-      </c>
-      <c r="E15" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="F15" s="37" t="s">
-        <v>88</v>
       </c>
       <c r="G15" s="15">
         <v>215.36</v>
       </c>
       <c r="H15" s="15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
@@ -1675,19 +1755,19 @@
         <v>1</v>
       </c>
       <c r="D16" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="F16" s="38" t="s">
         <v>87</v>
-      </c>
-      <c r="E16" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="F16" s="38" t="s">
-        <v>88</v>
       </c>
       <c r="G16" s="16">
         <v>171.08</v>
       </c>
       <c r="H16" s="16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
@@ -1701,19 +1781,19 @@
         <v>1</v>
       </c>
       <c r="D17" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="F17" s="39" t="s">
         <v>87</v>
-      </c>
-      <c r="E17" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="F17" s="39" t="s">
-        <v>88</v>
       </c>
       <c r="G17" s="17">
         <v>440.35</v>
       </c>
       <c r="H17" s="17" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
@@ -1727,19 +1807,19 @@
         <v>1</v>
       </c>
       <c r="D18" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="F18" s="40" t="s">
         <v>87</v>
-      </c>
-      <c r="E18" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="F18" s="40" t="s">
-        <v>88</v>
       </c>
       <c r="G18" s="18">
         <v>193.59</v>
       </c>
       <c r="H18" s="18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
@@ -1753,19 +1833,19 @@
         <v>1</v>
       </c>
       <c r="D19" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="E19" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="F19" s="41" t="s">
         <v>87</v>
-      </c>
-      <c r="E19" s="19" t="s">
-        <v>38</v>
-      </c>
-      <c r="F19" s="41" t="s">
-        <v>88</v>
       </c>
       <c r="G19" s="19">
         <v>100</v>
       </c>
       <c r="H19" s="19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
@@ -1779,19 +1859,19 @@
         <v>1</v>
       </c>
       <c r="D20" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="E20" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="F20" s="38" t="s">
         <v>87</v>
-      </c>
-      <c r="E20" s="20" t="s">
-        <v>38</v>
-      </c>
-      <c r="F20" s="38" t="s">
-        <v>88</v>
       </c>
       <c r="G20" s="20">
         <v>100</v>
       </c>
       <c r="H20" s="20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
@@ -1805,19 +1885,19 @@
         <v>1</v>
       </c>
       <c r="D21" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="E21" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="F21" s="39" t="s">
         <v>87</v>
-      </c>
-      <c r="E21" s="21" t="s">
-        <v>38</v>
-      </c>
-      <c r="F21" s="39" t="s">
-        <v>88</v>
       </c>
       <c r="G21" s="21">
         <v>100</v>
       </c>
       <c r="H21" s="21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
@@ -1831,19 +1911,19 @@
         <v>1</v>
       </c>
       <c r="D22" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="E22" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="F22" s="40" t="s">
         <v>87</v>
-      </c>
-      <c r="E22" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="F22" s="40" t="s">
-        <v>88</v>
       </c>
       <c r="G22" s="22">
         <v>100</v>
       </c>
       <c r="H22" s="22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
@@ -1857,29 +1937,134 @@
         <v>1</v>
       </c>
       <c r="D23" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="E23" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="F23" s="41" t="s">
         <v>87</v>
-      </c>
-      <c r="E23" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="F23" s="41" t="s">
-        <v>88</v>
       </c>
       <c r="G23" s="23">
         <v>100</v>
       </c>
       <c r="H23" s="23" t="s">
-        <v>39</v>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2">
+        <v>1</v>
+      </c>
+      <c r="C24" s="2">
+        <v>1</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="G24" s="2">
+        <v>100</v>
+      </c>
+      <c r="H24" s="24" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A25" s="3">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3">
+        <v>1</v>
+      </c>
+      <c r="C25" s="3">
+        <v>1</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F25" s="25" t="s">
+        <v>87</v>
+      </c>
+      <c r="G25" s="3">
+        <v>100</v>
+      </c>
+      <c r="H25" s="25" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A26" s="4">
+        <v>25</v>
+      </c>
+      <c r="B26" s="22">
+        <v>1</v>
+      </c>
+      <c r="C26" s="4">
+        <v>1</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F26" s="26" t="s">
+        <v>87</v>
+      </c>
+      <c r="G26" s="4">
+        <v>100</v>
+      </c>
+      <c r="H26" s="42" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A27" s="5">
+        <v>26</v>
+      </c>
+      <c r="B27" s="23">
+        <v>1</v>
+      </c>
+      <c r="C27" s="5">
+        <v>1</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="F27" s="27" t="s">
+        <v>87</v>
+      </c>
+      <c r="G27" s="5">
+        <v>100</v>
+      </c>
+      <c r="H27" s="43" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1900,22 +2085,22 @@
         <v>31</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
@@ -1926,22 +2111,22 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G2" s="2">
         <v>0.16</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
@@ -1952,22 +2137,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G3" s="3">
         <v>0</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
@@ -1978,22 +2163,22 @@
         <v>1</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G4" s="4">
         <v>0.16</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -2004,22 +2189,22 @@
         <v>1</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G5" s="4">
         <v>0</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
@@ -2030,22 +2215,22 @@
         <v>1</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G6" s="5">
         <v>0.53</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -2056,22 +2241,22 @@
         <v>1</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G7" s="5">
         <v>0.3</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
@@ -2082,22 +2267,22 @@
         <v>1</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G8" s="5">
         <v>0.26500000000000001</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
@@ -2108,22 +2293,22 @@
         <v>1</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G9" s="6">
         <v>0.16</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.35">
@@ -2134,22 +2319,22 @@
         <v>1</v>
       </c>
       <c r="C10" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D10" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>57</v>
-      </c>
       <c r="F10" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G10" s="6">
         <v>0.15</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
@@ -2160,22 +2345,22 @@
         <v>1</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G11" s="7">
         <v>0.16</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.35">
@@ -2186,22 +2371,22 @@
         <v>1</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G12" s="7">
         <v>0.53</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
@@ -2212,22 +2397,22 @@
         <v>1</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G13" s="7">
         <v>0.3</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
@@ -2238,22 +2423,22 @@
         <v>1</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G14" s="8">
         <v>0.16</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
@@ -2264,22 +2449,22 @@
         <v>1</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G15" s="8">
         <v>0</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
@@ -2290,22 +2475,22 @@
         <v>1</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G16" s="8">
         <v>0.08</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
@@ -2316,22 +2501,22 @@
         <v>1</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G17" s="9">
         <v>0.16</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
@@ -2342,22 +2527,22 @@
         <v>1</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G18" s="9">
         <v>0</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
@@ -2368,22 +2553,22 @@
         <v>1</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G19" s="9">
         <v>0.08</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.35">
@@ -2394,22 +2579,22 @@
         <v>1</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G20" s="9">
         <v>0.09</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.35">
@@ -2420,22 +2605,22 @@
         <v>1</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G21" s="10">
         <v>0.16</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
@@ -2446,22 +2631,22 @@
         <v>1</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G22" s="10">
         <v>0.16</v>
       </c>
       <c r="H22" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
@@ -2472,22 +2657,22 @@
         <v>1</v>
       </c>
       <c r="C23" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="E23" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="D23" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="E23" s="10" t="s">
-        <v>57</v>
-      </c>
       <c r="F23" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G23" s="10">
         <v>0.15</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
@@ -2498,22 +2683,22 @@
         <v>1</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D24" s="11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E24" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G24" s="11">
         <v>0.16</v>
       </c>
       <c r="H24" s="11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
@@ -2524,22 +2709,22 @@
         <v>1</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G25" s="11">
         <v>0</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
@@ -2550,22 +2735,22 @@
         <v>1</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E26" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G26" s="11">
         <v>0.09</v>
       </c>
       <c r="H26" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
@@ -2576,22 +2761,22 @@
         <v>1</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G27" s="11">
         <v>0.16</v>
       </c>
       <c r="H27" s="11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.35">
@@ -2602,22 +2787,22 @@
         <v>1</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E28" s="11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G28" s="11">
         <v>0.09</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.35">
@@ -2628,22 +2813,22 @@
         <v>1</v>
       </c>
       <c r="C29" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="D29" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="E29" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="D29" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="E29" s="11" t="s">
-        <v>57</v>
-      </c>
       <c r="F29" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G29" s="11">
         <v>0.16</v>
       </c>
       <c r="H29" s="11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
@@ -2654,22 +2839,22 @@
         <v>1</v>
       </c>
       <c r="C30" s="12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G30" s="12">
         <v>0.08</v>
       </c>
       <c r="H30" s="12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.35">
@@ -2680,22 +2865,22 @@
         <v>1</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F31" s="13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G31" s="13">
         <v>0.08</v>
       </c>
       <c r="H31" s="13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.35">
@@ -2706,22 +2891,22 @@
         <v>1</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F32" s="13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G32" s="13">
         <v>0</v>
       </c>
       <c r="H32" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.35">
@@ -2732,22 +2917,22 @@
         <v>1</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G33" s="14">
         <v>0.16</v>
       </c>
       <c r="H33" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.35">
@@ -2758,22 +2943,22 @@
         <v>1</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E34" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F34" s="14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G34" s="14">
         <v>0.08</v>
       </c>
       <c r="H34" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.35">
@@ -2784,22 +2969,22 @@
         <v>1</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G35" s="14">
         <v>0</v>
       </c>
       <c r="H35" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.35">
@@ -2810,22 +2995,22 @@
         <v>1</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E36" s="15" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F36" s="15" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G36" s="15">
         <v>0.08</v>
       </c>
       <c r="H36" s="15" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.35">
@@ -2836,22 +3021,22 @@
         <v>1</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E37" s="15" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F37" s="15" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G37" s="15">
         <v>0</v>
       </c>
       <c r="H37" s="15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.35">
@@ -2862,22 +3047,22 @@
         <v>1</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E38" s="15" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F38" s="15" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G38" s="15">
         <v>0.08</v>
       </c>
       <c r="H38" s="15" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.35">
@@ -2888,22 +3073,22 @@
         <v>1</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D39" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E39" s="15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F39" s="15" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G39" s="15">
         <v>0.08</v>
       </c>
       <c r="H39" s="15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.35">
@@ -2914,22 +3099,22 @@
         <v>1</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D40" s="15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E40" s="15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F40" s="15" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G40" s="15">
         <v>0.08</v>
       </c>
       <c r="H40" s="15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.35">
@@ -2940,22 +3125,22 @@
         <v>1</v>
       </c>
       <c r="C41" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="D41" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="D41" s="15" t="s">
-        <v>70</v>
-      </c>
       <c r="E41" s="15" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F41" s="15" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G41" s="15">
         <v>0.08</v>
       </c>
       <c r="H41" s="15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.35">
@@ -2966,22 +3151,22 @@
         <v>1</v>
       </c>
       <c r="C42" s="16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D42" s="16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E42" s="16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F42" s="16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G42" s="16">
         <v>0.16</v>
       </c>
       <c r="H42" s="16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.35">
@@ -2992,22 +3177,22 @@
         <v>1</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D43" s="16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E43" s="16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F43" s="16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G43" s="16">
         <v>0.09</v>
       </c>
       <c r="H43" s="16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.35">
@@ -3018,22 +3203,22 @@
         <v>1</v>
       </c>
       <c r="C44" s="16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D44" s="16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E44" s="16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F44" s="16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G44" s="16">
         <v>0.3</v>
       </c>
       <c r="H44" s="16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.35">
@@ -3044,22 +3229,22 @@
         <v>1</v>
       </c>
       <c r="C45" s="16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D45" s="16" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E45" s="16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F45" s="16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G45" s="16">
         <v>0.08</v>
       </c>
       <c r="H45" s="16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.35">
@@ -3070,22 +3255,22 @@
         <v>1</v>
       </c>
       <c r="C46" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="D46" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="D46" s="16" t="s">
-        <v>70</v>
-      </c>
       <c r="E46" s="16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F46" s="16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G46" s="16">
         <v>0.09</v>
       </c>
       <c r="H46" s="16" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.35">
@@ -3096,22 +3281,22 @@
         <v>1</v>
       </c>
       <c r="C47" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="D47" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="D47" s="16" t="s">
-        <v>70</v>
-      </c>
       <c r="E47" s="16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F47" s="16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G47" s="16">
         <v>0.08</v>
       </c>
       <c r="H47" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.35">
@@ -3122,22 +3307,22 @@
         <v>1</v>
       </c>
       <c r="C48" s="17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D48" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E48" s="17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F48" s="17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G48" s="17">
         <v>0.16</v>
       </c>
       <c r="H48" s="17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.35">
@@ -3148,22 +3333,22 @@
         <v>1</v>
       </c>
       <c r="C49" s="17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D49" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E49" s="17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F49" s="17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G49" s="17">
         <v>0.08</v>
       </c>
       <c r="H49" s="17" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.35">
@@ -3174,22 +3359,22 @@
         <v>1</v>
       </c>
       <c r="C50" s="17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D50" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E50" s="17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F50" s="17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G50" s="17">
         <v>0</v>
       </c>
       <c r="H50" s="17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.35">
@@ -3200,22 +3385,22 @@
         <v>1</v>
       </c>
       <c r="C51" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D51" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E51" s="17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F51" s="17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G51" s="17">
         <v>0.08</v>
       </c>
       <c r="H51" s="17" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.35">
@@ -3226,22 +3411,22 @@
         <v>1</v>
       </c>
       <c r="C52" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D52" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E52" s="17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F52" s="17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G52" s="17">
         <v>0.53</v>
       </c>
       <c r="H52" s="17" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.35">
@@ -3252,22 +3437,22 @@
         <v>1</v>
       </c>
       <c r="C53" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D53" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E53" s="17" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F53" s="17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G53" s="17">
         <v>0.3</v>
       </c>
       <c r="H53" s="17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.35">
@@ -3278,22 +3463,22 @@
         <v>1</v>
       </c>
       <c r="C54" s="18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D54" s="18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E54" s="18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F54" s="18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G54" s="18">
         <v>0.08</v>
       </c>
       <c r="H54" s="18" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.35">
@@ -3304,22 +3489,22 @@
         <v>1</v>
       </c>
       <c r="C55" s="18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D55" s="18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E55" s="18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F55" s="18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G55" s="18">
         <v>0</v>
       </c>
       <c r="H55" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.35">
@@ -3330,22 +3515,22 @@
         <v>1</v>
       </c>
       <c r="C56" s="18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D56" s="18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E56" s="18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F56" s="18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G56" s="18">
         <v>0.08</v>
       </c>
       <c r="H56" s="18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.35">
@@ -3356,22 +3541,22 @@
         <v>1</v>
       </c>
       <c r="C57" s="18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D57" s="18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E57" s="18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F57" s="18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G57" s="18">
         <v>0.53</v>
       </c>
       <c r="H57" s="18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.35">
@@ -3382,22 +3567,22 @@
         <v>1</v>
       </c>
       <c r="C58" s="18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D58" s="18" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E58" s="18" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F58" s="18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G58" s="18">
         <v>0.08</v>
       </c>
       <c r="H58" s="18" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.35">
@@ -3408,22 +3593,22 @@
         <v>1</v>
       </c>
       <c r="C59" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="D59" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="D59" s="18" t="s">
-        <v>70</v>
-      </c>
       <c r="E59" s="18" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F59" s="18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G59" s="18">
         <v>0.08</v>
       </c>
       <c r="H59" s="18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.35">
@@ -3434,22 +3619,22 @@
         <v>1</v>
       </c>
       <c r="C60" s="19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D60" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E60" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F60" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G60" s="19">
         <v>0.16</v>
       </c>
       <c r="H60" s="19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.35">
@@ -3460,22 +3645,22 @@
         <v>1</v>
       </c>
       <c r="C61" s="19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D61" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E61" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F61" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G61" s="19">
         <v>0.08</v>
       </c>
       <c r="H61" s="19" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.35">
@@ -3486,22 +3671,22 @@
         <v>1</v>
       </c>
       <c r="C62" s="19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D62" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E62" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F62" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G62" s="19">
         <v>0</v>
       </c>
       <c r="H62" s="19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.35">
@@ -3512,22 +3697,22 @@
         <v>1</v>
       </c>
       <c r="C63" s="19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D63" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E63" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F63" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G63" s="19">
         <v>0.08</v>
       </c>
       <c r="H63" s="19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.35">
@@ -3538,22 +3723,22 @@
         <v>1</v>
       </c>
       <c r="C64" s="19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D64" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E64" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F64" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G64" s="19">
         <v>0.53</v>
       </c>
       <c r="H64" s="19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.35">
@@ -3564,22 +3749,22 @@
         <v>1</v>
       </c>
       <c r="C65" s="19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D65" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E65" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F65" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G65" s="19">
         <v>0.26500000000000001</v>
       </c>
       <c r="H65" s="19" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.35">
@@ -3590,22 +3775,22 @@
         <v>1</v>
       </c>
       <c r="C66" s="19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D66" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E66" s="19" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F66" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G66" s="19">
         <v>0.08</v>
       </c>
       <c r="H66" s="19" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.35">
@@ -3616,22 +3801,22 @@
         <v>1</v>
       </c>
       <c r="C67" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="D67" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="E67" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="D67" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="E67" s="19" t="s">
-        <v>57</v>
-      </c>
       <c r="F67" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G67" s="19">
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="H67" s="19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.35">
@@ -3642,22 +3827,22 @@
         <v>1</v>
       </c>
       <c r="C68" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="D68" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="D68" s="19" t="s">
-        <v>70</v>
-      </c>
       <c r="E68" s="19" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F68" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G68" s="19">
         <v>0.05</v>
       </c>
       <c r="H68" s="19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.35">
@@ -3668,22 +3853,22 @@
         <v>1</v>
       </c>
       <c r="C69" s="20" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D69" s="20" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E69" s="20" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F69" s="20" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G69" s="20">
         <v>0.16</v>
       </c>
       <c r="H69" s="20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.35">
@@ -3694,22 +3879,22 @@
         <v>1</v>
       </c>
       <c r="C70" s="21" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D70" s="21" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E70" s="21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F70" s="21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G70" s="21">
         <v>0.16</v>
       </c>
       <c r="H70" s="21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.35">
@@ -3720,22 +3905,22 @@
         <v>1</v>
       </c>
       <c r="C71" s="22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D71" s="22" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E71" s="22" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F71" s="22" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G71" s="22">
         <v>0.16</v>
       </c>
       <c r="H71" s="22" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.35">
@@ -3746,22 +3931,22 @@
         <v>1</v>
       </c>
       <c r="C72" s="22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D72" s="22" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E72" s="22" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F72" s="22" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G72" s="22">
         <v>0</v>
       </c>
       <c r="H72" s="22" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.35">
@@ -3772,22 +3957,22 @@
         <v>1</v>
       </c>
       <c r="C73" s="22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D73" s="22" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E73" s="22" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F73" s="22" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G73" s="22">
         <v>0.08</v>
       </c>
       <c r="H73" s="22" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.35">
@@ -3798,22 +3983,22 @@
         <v>1</v>
       </c>
       <c r="C74" s="22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D74" s="22" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E74" s="22" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F74" s="22" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G74" s="22">
         <v>0.09</v>
       </c>
       <c r="H74" s="22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.35">
@@ -3824,22 +4009,126 @@
         <v>1</v>
       </c>
       <c r="C75" s="23" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E75" s="23" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F75" s="23" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G75" s="23">
         <v>0.16</v>
       </c>
       <c r="H75" s="23" t="s">
-        <v>50</v>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A76" s="2">
+        <v>23</v>
+      </c>
+      <c r="B76" s="2">
+        <v>1</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G76" s="2">
+        <v>0.16</v>
+      </c>
+      <c r="H76" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A77" s="3">
+        <v>24</v>
+      </c>
+      <c r="B77" s="3">
+        <v>1</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E77" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="F77" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G77" s="3">
+        <v>0.16</v>
+      </c>
+      <c r="H77" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A78" s="4">
+        <v>25</v>
+      </c>
+      <c r="B78" s="4">
+        <v>1</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D78" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E78" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="F78" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="G78" s="4">
+        <v>0.16</v>
+      </c>
+      <c r="H78" s="22" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A79" s="5">
+        <v>26</v>
+      </c>
+      <c r="B79" s="5">
+        <v>1</v>
+      </c>
+      <c r="C79" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D79" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E79" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="F79" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="G79" s="5">
+        <v>0.16</v>
+      </c>
+      <c r="H79" s="23" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -3849,7 +4138,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -3862,44 +4151,53 @@
     <col min="10" max="10" width="10.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" s="2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>85</v>
       </c>
       <c r="E2" s="2">
         <v>0</v>
@@ -3913,19 +4211,22 @@
       <c r="H2" s="2">
         <v>41</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>84</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>85</v>
       </c>
       <c r="E3" s="3">
         <v>0</v>
@@ -3939,19 +4240,22 @@
       <c r="H3" s="3">
         <v>25</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>84</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>85</v>
       </c>
       <c r="E4" s="4">
         <v>0</v>
@@ -3965,19 +4269,22 @@
       <c r="H4" s="4">
         <v>41</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I4" s="4"/>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>84</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>85</v>
       </c>
       <c r="E5" s="5">
         <v>0</v>
@@ -3991,19 +4298,22 @@
       <c r="H5" s="5">
         <v>109.5</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" s="6">
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>84</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>85</v>
       </c>
       <c r="E6" s="6">
         <v>0</v>
@@ -4015,21 +4325,24 @@
         <v>100</v>
       </c>
       <c r="H6" s="6">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="I6" s="6"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" s="7">
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="D7" s="7" t="s">
         <v>84</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>85</v>
       </c>
       <c r="E7" s="7">
         <v>0</v>
@@ -4041,21 +4354,24 @@
         <v>80</v>
       </c>
       <c r="H7" s="7">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+        <v>21.48</v>
+      </c>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="8">
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="D8" s="8" t="s">
         <v>84</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>85</v>
       </c>
       <c r="E8" s="8">
         <v>0</v>
@@ -4069,19 +4385,22 @@
       <c r="H8" s="8">
         <v>56.433300000000003</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="9">
         <v>8</v>
       </c>
       <c r="B9" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="D9" s="9" t="s">
         <v>84</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>85</v>
       </c>
       <c r="E9" s="9">
         <v>0</v>
@@ -4095,19 +4414,22 @@
       <c r="H9" s="9">
         <v>84.000100000000003</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" s="10">
         <v>9</v>
       </c>
       <c r="B10" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="C10" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="D10" s="10" t="s">
         <v>84</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>85</v>
       </c>
       <c r="E10" s="10">
         <v>0</v>
@@ -4119,21 +4441,24 @@
         <v>251</v>
       </c>
       <c r="H10" s="10">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+        <v>46.5</v>
+      </c>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="11">
         <v>10</v>
       </c>
       <c r="B11" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="C11" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="D11" s="11" t="s">
         <v>84</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>85</v>
       </c>
       <c r="E11" s="11">
         <v>0</v>
@@ -4145,21 +4470,24 @@
         <v>38.756435000000003</v>
       </c>
       <c r="H11" s="11">
-        <v>86.243565000000004</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+        <v>45.236848000000002</v>
+      </c>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" s="12">
         <v>11</v>
       </c>
       <c r="B12" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C12" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="D12" s="12" t="s">
         <v>84</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>85</v>
       </c>
       <c r="E12" s="12">
         <v>0</v>
@@ -4173,19 +4501,22 @@
       <c r="H12" s="12">
         <v>36.456598</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="12"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" s="13">
         <v>12</v>
       </c>
       <c r="B13" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C13" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="D13" s="13" t="s">
         <v>84</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>85</v>
       </c>
       <c r="E13" s="13">
         <v>0</v>
@@ -4199,19 +4530,22 @@
       <c r="H13" s="13">
         <v>36.456598</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I13" s="13"/>
+      <c r="J13" s="13"/>
+      <c r="K13" s="13"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" s="14">
         <v>13</v>
       </c>
       <c r="B14" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="D14" s="14" t="s">
         <v>84</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>85</v>
       </c>
       <c r="E14" s="14">
         <v>0</v>
@@ -4223,21 +4557,24 @@
         <v>44.42</v>
       </c>
       <c r="H14" s="14">
-        <v>133.01</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+        <v>101.19</v>
+      </c>
+      <c r="I14" s="14"/>
+      <c r="J14" s="14"/>
+      <c r="K14" s="14"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" s="15">
         <v>14</v>
       </c>
       <c r="B15" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="D15" s="15" t="s">
         <v>84</v>
-      </c>
-      <c r="D15" s="15" t="s">
-        <v>85</v>
       </c>
       <c r="E15" s="15">
         <v>0</v>
@@ -4251,19 +4588,22 @@
       <c r="H15" s="15">
         <v>100.2</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I15" s="15"/>
+      <c r="J15" s="15"/>
+      <c r="K15" s="15"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" s="16">
         <v>15</v>
       </c>
       <c r="B16" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="D16" s="16" t="s">
         <v>84</v>
-      </c>
-      <c r="D16" s="16" t="s">
-        <v>85</v>
       </c>
       <c r="E16" s="16">
         <v>0</v>
@@ -4277,19 +4617,22 @@
       <c r="H16" s="16">
         <v>101</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="16"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" s="17">
         <v>16</v>
       </c>
       <c r="B17" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="C17" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="D17" s="17" t="s">
         <v>84</v>
-      </c>
-      <c r="D17" s="17" t="s">
-        <v>85</v>
       </c>
       <c r="E17" s="17">
         <v>0</v>
@@ -4303,19 +4646,22 @@
       <c r="H17" s="17">
         <v>220.17500000000001</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="17"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="18">
         <v>17</v>
       </c>
       <c r="B18" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="C18" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="D18" s="18" t="s">
         <v>84</v>
-      </c>
-      <c r="D18" s="18" t="s">
-        <v>85</v>
       </c>
       <c r="E18" s="18">
         <v>0</v>
@@ -4329,20 +4675,22 @@
       <c r="H18" s="18">
         <v>100</v>
       </c>
-      <c r="J18" s="42"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I18" s="18"/>
+      <c r="J18" s="18"/>
+      <c r="K18" s="18"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" s="19">
         <v>18</v>
       </c>
       <c r="B19" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="C19" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="D19" s="19" t="s">
         <v>84</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>85</v>
       </c>
       <c r="E19" s="19">
         <v>0</v>
@@ -4356,16 +4704,19 @@
       <c r="H19" s="19">
         <v>98.92</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I19" s="19"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" s="20">
         <v>19</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D20" s="20" t="s">
         <v>29</v>
@@ -4382,16 +4733,19 @@
       <c r="H20" s="20">
         <v>0.625</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I20" s="20"/>
+      <c r="J20" s="20"/>
+      <c r="K20" s="20"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" s="21">
         <v>20</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D21" s="21" t="s">
         <v>29</v>
@@ -4408,19 +4762,22 @@
       <c r="H21" s="21">
         <v>0.625</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I21" s="21"/>
+      <c r="J21" s="21"/>
+      <c r="K21" s="21"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" s="22">
         <v>21</v>
       </c>
       <c r="B22" s="22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E22" s="22">
         <v>17.5</v>
@@ -4434,19 +4791,22 @@
       <c r="H22" s="22">
         <v>875</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I22" s="22"/>
+      <c r="J22" s="22"/>
+      <c r="K22" s="22"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" s="23">
         <v>22</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E23" s="23">
         <v>17.5</v>
@@ -4460,8 +4820,128 @@
       <c r="H23" s="23">
         <v>875</v>
       </c>
+      <c r="I23" s="23"/>
+      <c r="J23" s="23"/>
+      <c r="K23" s="23"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E24" s="2">
+        <v>20</v>
+      </c>
+      <c r="F24" s="2">
+        <v>20</v>
+      </c>
+      <c r="G24" s="2">
+        <v>5</v>
+      </c>
+      <c r="H24" s="2">
+        <v>0.8</v>
+      </c>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A25" s="3">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E25" s="3">
+        <v>17.460317</v>
+      </c>
+      <c r="F25" s="3">
+        <v>17.460317</v>
+      </c>
+      <c r="G25" s="3">
+        <v>6</v>
+      </c>
+      <c r="H25" s="3">
+        <v>0.64</v>
+      </c>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A26" s="4">
+        <v>25</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E26" s="4">
+        <v>17.5</v>
+      </c>
+      <c r="F26" s="4">
+        <v>17.5</v>
+      </c>
+      <c r="G26" s="4">
+        <v>6</v>
+      </c>
+      <c r="H26" s="4">
+        <v>0.63</v>
+      </c>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A27" s="5">
+        <v>26</v>
+      </c>
+      <c r="B27" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="E27" s="5">
+        <v>0</v>
+      </c>
+      <c r="F27" s="5">
+        <v>0</v>
+      </c>
+      <c r="G27" s="5">
+        <v>75</v>
+      </c>
+      <c r="H27" s="23">
+        <v>41</v>
+      </c>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="5"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>